<commit_message>
Move new application refusers to membership import
</commit_message>
<xml_diff>
--- a/output/20260630_fix_owner_new_import/active_problem_1_no_payment_cash_3_cases_20260630.xlsx
+++ b/output/20260630_fix_owner_new_import/active_problem_1_no_payment_cash_3_cases_20260630.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Импорт_абонементы" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Импорт_абонементы'!$A$1:$T$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Импорт_абонементы'!$A$1:$U$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -435,170 +435,174 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T4"/>
+  <dimension ref="A1:U4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
     <col width="21" customWidth="1" min="10" max="10"/>
     <col width="21" customWidth="1" min="11" max="11"/>
     <col width="21" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="21" customWidth="1" min="13" max="13"/>
     <col width="10" customWidth="1" min="14" max="14"/>
-    <col width="13" customWidth="1" min="15" max="15"/>
-    <col width="10" customWidth="1" min="16" max="16"/>
-    <col width="20" customWidth="1" min="17" max="17"/>
-    <col width="14" customWidth="1" min="18" max="18"/>
-    <col width="17" customWidth="1" min="19" max="19"/>
-    <col width="34" customWidth="1" min="20" max="20"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="10" customWidth="1" min="17" max="17"/>
+    <col width="20" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="17" customWidth="1" min="20" max="20"/>
+    <col width="34" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>tag</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>contract_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>client_id</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>phone</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>client_fio</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>contract_name</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>card</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>duration</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>duration_type</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>create_date</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>payment_date</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>activation_date</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>end_date</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>freeze</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>guests</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>visits_left</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>price</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>amount_of_payments</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>payment_left</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>type_of_payment</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>manager</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>00000150603</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>000009536</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>+7 (921) 6274391</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Куфтарева Зоя Викторовна</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Абонемент МУЛЬТИКАРТА 12 месяцев + подарок (СПЕЦПРЕДЛОЖЕНИЕ)</t>
         </is>
       </c>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n">
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>месяц</t>
         </is>
-      </c>
-      <c r="I2" s="3" t="n">
-        <v>46165</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>46165</v>
@@ -607,183 +611,188 @@
         <v>46165</v>
       </c>
       <c r="L2" s="3" t="n">
+        <v>46165</v>
+      </c>
+      <c r="M2" s="3" t="n">
         <v>46529</v>
       </c>
-      <c r="M2" s="2" t="n">
+      <c r="N2" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="N2" s="2" t="n"/>
       <c r="O2" s="2" t="n"/>
-      <c r="P2" s="2" t="n">
-        <v>11990</v>
-      </c>
+      <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="n">
         <v>11990</v>
       </c>
       <c r="R2" s="2" t="n">
+        <v>11990</v>
+      </c>
+      <c r="S2" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="S2" s="2" t="inlineStr">
+      <c r="T2" s="2" t="inlineStr">
         <is>
           <t>наличные</t>
         </is>
       </c>
-      <c r="T2" s="2" t="inlineStr">
+      <c r="U2" s="2" t="inlineStr">
         <is>
           <t>Васильева Яна Денисовна</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="2" t="n"/>
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>00000147835</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>000072532</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>+7 (953) 5474369</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Лукина Варвара Сергеевна</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Абонемент УЛЬТРА 12 месяцев</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>000010012628</t>
         </is>
       </c>
-      <c r="G3" s="2" t="n">
+      <c r="H3" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>месяц</t>
         </is>
       </c>
-      <c r="I3" s="3" t="n">
+      <c r="J3" s="3" t="n">
         <v>46062</v>
       </c>
-      <c r="J3" s="3" t="n">
+      <c r="K3" s="3" t="n">
         <v>46090</v>
       </c>
-      <c r="K3" s="3" t="n">
+      <c r="L3" s="3" t="n">
         <v>46086</v>
       </c>
-      <c r="L3" s="3" t="n">
+      <c r="M3" s="3" t="n">
         <v>46450</v>
       </c>
-      <c r="M3" s="2" t="n"/>
       <c r="N3" s="2" t="n"/>
       <c r="O3" s="2" t="n"/>
-      <c r="P3" s="2" t="n">
-        <v>14990</v>
-      </c>
+      <c r="P3" s="2" t="n"/>
       <c r="Q3" s="2" t="n">
         <v>14990</v>
       </c>
       <c r="R3" s="2" t="n">
+        <v>14990</v>
+      </c>
+      <c r="S3" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="S3" s="2" t="inlineStr">
+      <c r="T3" s="2" t="inlineStr">
         <is>
           <t>наличные</t>
         </is>
       </c>
-      <c r="T3" s="2" t="inlineStr">
+      <c r="U3" s="2" t="inlineStr">
         <is>
           <t>Соколова Анастасия Александровна</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="2" t="n"/>
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>00000145604</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>000027130</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>+7 (911) 4050018</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Мамай Анастасия Витальевна</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>Абонемент МУЛЬТИКАРТА 12 месяцев СПЕЦПРЕДЛОЖЕНИЕ</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>115000151321</t>
         </is>
       </c>
-      <c r="G4" s="2" t="n">
+      <c r="H4" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>месяц</t>
         </is>
       </c>
-      <c r="I4" s="3" t="n">
+      <c r="J4" s="3" t="n">
         <v>45213</v>
-      </c>
-      <c r="J4" s="3" t="n">
-        <v>46039</v>
       </c>
       <c r="K4" s="3" t="n">
         <v>46039</v>
       </c>
       <c r="L4" s="3" t="n">
+        <v>46039</v>
+      </c>
+      <c r="M4" s="3" t="n">
         <v>46403</v>
       </c>
-      <c r="M4" s="2" t="n"/>
       <c r="N4" s="2" t="n"/>
       <c r="O4" s="2" t="n"/>
-      <c r="P4" s="2" t="n">
-        <v>11990</v>
-      </c>
+      <c r="P4" s="2" t="n"/>
       <c r="Q4" s="2" t="n">
         <v>11990</v>
       </c>
       <c r="R4" s="2" t="n">
+        <v>11990</v>
+      </c>
+      <c r="S4" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="S4" s="2" t="inlineStr">
+      <c r="T4" s="2" t="inlineStr">
         <is>
           <t>наличные</t>
         </is>
       </c>
-      <c r="T4" s="2" t="inlineStr">
+      <c r="U4" s="2" t="inlineStr">
         <is>
           <t>Петрова Полина Владимировна</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T4"/>
+  <autoFilter ref="A1:U4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>